<commit_message>
Dodaje walidację ciągłości flag F/G w oknie 12 miesięcy (zadanie 1.4)
Nowy moduł validateFlagContinuity.ts: dla każdego NIP sprawdza, czy
flaga F/G jest spójna z historią dostępu klienta (SPEC.md II.3.g) -
F wymaga przerwy >12 miesięcy od poprzedniego dostępu (lub braku
historii), G wymaga przerwy <=12 miesięcy, z regułą horyzontu dla G
bez widocznej historii w pierwszych 12 miesiącach danych. Flaga I
(i H) wykluczona z łańcucha ciągłości - potwierdzone empirycznie na
danych syntetycznych (SPEC.md V.28).

Ta sama analiza ujawniła błąd w scripts/generate-synthetic-data.ts:
przerwa między pakietami liczona była od końca ostatniego wersu
w ogóle (także incydentalnych), zamiast od końca ostatniego
prawdziwego dostępu F/G. Naprawiono generator i przegenerowano oba
pliki syntetyczne (ta sama liczba wersów, poprawione flagi w 22
wersach pliku czystego).
</commit_message>
<xml_diff>
--- a/test-data/dane-syntetyczne-clean.xlsx
+++ b/test-data/dane-syntetyczne-clean.xlsx
@@ -3928,7 +3928,7 @@
       <c r="E79">
         <v>30207.36</v>
       </c>
-      <c r="G79">
+      <c r="F79">
         <v>1</v>
       </c>
       <c r="M79">
@@ -6227,7 +6227,7 @@
       <c r="E135">
         <v>30844.2</v>
       </c>
-      <c r="G135">
+      <c r="F135">
         <v>1</v>
       </c>
       <c r="N135">
@@ -8353,7 +8353,7 @@
       <c r="E184">
         <v>11997.6</v>
       </c>
-      <c r="G184">
+      <c r="F184">
         <v>1</v>
       </c>
       <c r="P184">
@@ -9714,7 +9714,7 @@
       <c r="E215">
         <v>28286</v>
       </c>
-      <c r="G215">
+      <c r="F215">
         <v>1</v>
       </c>
       <c r="Q215">
@@ -10448,7 +10448,7 @@
       <c r="E231">
         <v>34337.71</v>
       </c>
-      <c r="G231">
+      <c r="F231">
         <v>1</v>
       </c>
       <c r="R231">
@@ -13142,7 +13142,7 @@
       <c r="E294">
         <v>11798.16</v>
       </c>
-      <c r="G294">
+      <c r="F294">
         <v>1</v>
       </c>
       <c r="T294">
@@ -13577,7 +13577,7 @@
       <c r="E303">
         <v>37076.16</v>
       </c>
-      <c r="G303">
+      <c r="F303">
         <v>1</v>
       </c>
       <c r="T303">
@@ -13885,7 +13885,7 @@
       <c r="E310">
         <v>14418.8</v>
       </c>
-      <c r="G310">
+      <c r="F310">
         <v>1</v>
       </c>
       <c r="T310">
@@ -15488,7 +15488,7 @@
       <c r="E345">
         <v>75619.92</v>
       </c>
-      <c r="G345">
+      <c r="F345">
         <v>1</v>
       </c>
       <c r="U345">
@@ -16943,7 +16943,7 @@
       <c r="E375">
         <v>25770.36</v>
       </c>
-      <c r="G375">
+      <c r="F375">
         <v>1</v>
       </c>
       <c r="V375">
@@ -17055,7 +17055,7 @@
       <c r="E377">
         <v>30909.84</v>
       </c>
-      <c r="G377">
+      <c r="F377">
         <v>1</v>
       </c>
       <c r="V377">
@@ -19656,7 +19656,7 @@
       <c r="E437">
         <v>76224.72</v>
       </c>
-      <c r="G437">
+      <c r="F437">
         <v>1</v>
       </c>
       <c r="X437">
@@ -20400,7 +20400,7 @@
       <c r="E452">
         <v>16712.16</v>
       </c>
-      <c r="G452">
+      <c r="F452">
         <v>1</v>
       </c>
       <c r="X452">
@@ -21664,7 +21664,7 @@
       <c r="E478">
         <v>11340.12</v>
       </c>
-      <c r="G478">
+      <c r="F478">
         <v>1</v>
       </c>
       <c r="Y478">
@@ -24550,7 +24550,7 @@
       <c r="E538">
         <v>13118.88</v>
       </c>
-      <c r="G538">
+      <c r="F538">
         <v>1</v>
       </c>
       <c r="Z538">
@@ -25881,7 +25881,7 @@
       <c r="E569">
         <v>30489.24</v>
       </c>
-      <c r="G569">
+      <c r="F569">
         <v>1</v>
       </c>
       <c r="AA569">
@@ -26322,7 +26322,7 @@
       <c r="E578">
         <v>35256.48</v>
       </c>
-      <c r="G578">
+      <c r="F578">
         <v>1</v>
       </c>
       <c r="AA578">
@@ -27160,7 +27160,7 @@
       <c r="E595">
         <v>34885.56</v>
       </c>
-      <c r="G595">
+      <c r="F595">
         <v>1</v>
       </c>
       <c r="AB595">
@@ -31941,7 +31941,7 @@
       <c r="E698">
         <v>10756.56</v>
       </c>
-      <c r="G698">
+      <c r="F698">
         <v>1</v>
       </c>
       <c r="AD698">
@@ -32742,7 +32742,7 @@
       <c r="E713">
         <v>15381.24</v>
       </c>
-      <c r="G713">
+      <c r="F713">
         <v>1</v>
       </c>
       <c r="AD713">
@@ -33793,7 +33793,7 @@
       <c r="E736">
         <v>25616.88</v>
       </c>
-      <c r="G736">
+      <c r="F736">
         <v>1</v>
       </c>
       <c r="AE736">
@@ -37965,7 +37965,7 @@
       <c r="E824">
         <v>32075.28</v>
       </c>
-      <c r="G824">
+      <c r="F824">
         <v>1</v>
       </c>
       <c r="AG824">
@@ -38077,7 +38077,7 @@
       <c r="E826">
         <v>26229.6</v>
       </c>
-      <c r="G826">
+      <c r="F826">
         <v>1</v>
       </c>
       <c r="AG826">
@@ -38261,7 +38261,7 @@
       <c r="E831">
         <v>44434.32</v>
       </c>
-      <c r="G831">
+      <c r="F831">
         <v>1</v>
       </c>
       <c r="AG831">
@@ -39312,7 +39312,7 @@
       <c r="E854">
         <v>12877.56</v>
       </c>
-      <c r="G854">
+      <c r="F854">
         <v>1</v>
       </c>
       <c r="AH854">
@@ -39794,7 +39794,7 @@
       <c r="E864">
         <v>27654.24</v>
       </c>
-      <c r="G864">
+      <c r="F864">
         <v>1</v>
       </c>
       <c r="AH864">
@@ -41089,7 +41089,7 @@
       <c r="E895">
         <v>89069.76</v>
       </c>
-      <c r="G895">
+      <c r="F895">
         <v>1</v>
       </c>
       <c r="AH895">
@@ -42406,7 +42406,7 @@
       <c r="E922">
         <v>12252.12</v>
       </c>
-      <c r="G922">
+      <c r="F922">
         <v>1</v>
       </c>
       <c r="AI922">
@@ -44880,7 +44880,7 @@
       <c r="E977">
         <v>29370.12</v>
       </c>
-      <c r="G977">
+      <c r="F977">
         <v>1</v>
       </c>
       <c r="AK977">
@@ -44959,7 +44959,7 @@
       <c r="E979">
         <v>43674.96</v>
       </c>
-      <c r="G979">
+      <c r="F979">
         <v>1</v>
       </c>
       <c r="AK979">
@@ -46191,7 +46191,7 @@
       <c r="E1007">
         <v>23784.6</v>
       </c>
-      <c r="G1007">
+      <c r="F1007">
         <v>1</v>
       </c>
       <c r="AK1007">

</xml_diff>

<commit_message>
Koryguje rozkład miesięczny korekt FKS na zasadę nieretroaktywności ksiąg
Korekta nie może zmieniać już zrealizowanych (zamkniętych) miesięcy - ich
reversal ujmowany jest w całości w miesiącu sprzedaży samej korekty, nie
wraca do przeszłości. Poprawiono generator danych syntetycznych (wcześniej
naiwnie negował oryginalny rozkład miesięczny), oba pliki przegenerowane.
Decyzja opisana w SPEC.md V.33.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-data/dane-syntetyczne-clean.xlsx
+++ b/test-data/dane-syntetyczne-clean.xlsx
@@ -1441,11 +1441,8 @@
       <c r="E25">
         <v>-38905.2</v>
       </c>
-      <c r="J25">
-        <v>-3242.1</v>
-      </c>
       <c r="K25">
-        <v>-3242.1</v>
+        <v>-6484.2</v>
       </c>
       <c r="L25">
         <v>-3242.1</v>
@@ -1494,7 +1491,7 @@
       <c r="E26">
         <v>-9583.19</v>
       </c>
-      <c r="J26">
+      <c r="K26">
         <v>-9583.19</v>
       </c>
     </row>
@@ -2526,7 +2523,7 @@
       <c r="E47">
         <v>-28327.57</v>
       </c>
-      <c r="K47">
+      <c r="L47">
         <v>-28327.57</v>
       </c>
     </row>
@@ -3690,11 +3687,8 @@
       <c r="E74">
         <v>-43766.88</v>
       </c>
-      <c r="L74">
-        <v>-3647.24</v>
-      </c>
       <c r="M74">
-        <v>-3647.24</v>
+        <v>-7294.48</v>
       </c>
       <c r="N74">
         <v>-3647.24</v>
@@ -3743,11 +3737,8 @@
       <c r="E75">
         <v>-15948.24</v>
       </c>
-      <c r="L75">
-        <v>-1329.02</v>
-      </c>
       <c r="M75">
-        <v>-1329.02</v>
+        <v>-2658.04</v>
       </c>
       <c r="N75">
         <v>-1329.02</v>
@@ -3796,14 +3787,8 @@
       <c r="E76">
         <v>-34014.24</v>
       </c>
-      <c r="K76">
-        <v>-2834.52</v>
-      </c>
-      <c r="L76">
-        <v>-2834.52</v>
-      </c>
       <c r="M76">
-        <v>-2834.52</v>
+        <v>-8503.56</v>
       </c>
       <c r="N76">
         <v>-2834.52</v>
@@ -4850,11 +4835,8 @@
       <c r="E102">
         <v>-25960.32</v>
       </c>
-      <c r="M102">
-        <v>-2163.36</v>
-      </c>
       <c r="N102">
-        <v>-2163.36</v>
+        <v>-4326.72</v>
       </c>
       <c r="O102">
         <v>-2163.36</v>
@@ -4903,14 +4885,8 @@
       <c r="E103">
         <v>-14400</v>
       </c>
-      <c r="L103">
-        <v>-1200</v>
-      </c>
-      <c r="M103">
-        <v>-1200</v>
-      </c>
       <c r="N103">
-        <v>-1200</v>
+        <v>-3600</v>
       </c>
       <c r="O103">
         <v>-1200</v>
@@ -4956,7 +4932,7 @@
       <c r="E104">
         <v>-8198.23</v>
       </c>
-      <c r="L104">
+      <c r="N104">
         <v>-8198.23</v>
       </c>
     </row>
@@ -7842,7 +7818,7 @@
       <c r="E173">
         <v>-18485.26</v>
       </c>
-      <c r="O173">
+      <c r="P173">
         <v>-18485.26</v>
       </c>
     </row>
@@ -9047,11 +9023,8 @@
       <c r="E198">
         <v>-3384.45</v>
       </c>
-      <c r="P198">
-        <v>-676.89</v>
-      </c>
       <c r="Q198">
-        <v>-676.89</v>
+        <v>-1353.78</v>
       </c>
       <c r="R198">
         <v>-676.89</v>
@@ -11326,14 +11299,8 @@
       <c r="E250">
         <v>-14023.44</v>
       </c>
-      <c r="Q250">
-        <v>-1168.62</v>
-      </c>
-      <c r="R250">
-        <v>-1168.62</v>
-      </c>
       <c r="S250">
-        <v>-1168.62</v>
+        <v>-3505.86</v>
       </c>
       <c r="T250">
         <v>-1168.62</v>
@@ -12686,11 +12653,8 @@
       <c r="E282">
         <v>-2839.5</v>
       </c>
-      <c r="S282">
-        <v>-473.25</v>
-      </c>
       <c r="T282">
-        <v>-473.25</v>
+        <v>-946.5</v>
       </c>
       <c r="U282">
         <v>-473.25</v>
@@ -14153,14 +14117,8 @@
       <c r="E315">
         <v>-9706.92</v>
       </c>
-      <c r="S315">
-        <v>-808.91</v>
-      </c>
-      <c r="T315">
-        <v>-808.91</v>
-      </c>
       <c r="U315">
-        <v>-808.91</v>
+        <v>-2426.73</v>
       </c>
       <c r="V315">
         <v>-808.91</v>
@@ -14206,11 +14164,8 @@
       <c r="E316">
         <v>-45267</v>
       </c>
-      <c r="T316">
-        <v>-3772.25</v>
-      </c>
       <c r="U316">
-        <v>-3772.25</v>
+        <v>-7544.5</v>
       </c>
       <c r="V316">
         <v>-3772.25</v>
@@ -15918,7 +15873,7 @@
       <c r="E353">
         <v>-7591.63</v>
       </c>
-      <c r="U353">
+      <c r="V353">
         <v>-7591.63</v>
       </c>
     </row>
@@ -15938,14 +15893,8 @@
       <c r="E354">
         <v>-2042.46</v>
       </c>
-      <c r="T354">
-        <v>-680.82</v>
-      </c>
-      <c r="U354">
-        <v>-680.82</v>
-      </c>
       <c r="V354">
-        <v>-680.82</v>
+        <v>-2042.46</v>
       </c>
     </row>
     <row r="355">
@@ -15964,11 +15913,8 @@
       <c r="E355">
         <v>-2748.48</v>
       </c>
-      <c r="U355">
-        <v>-343.56</v>
-      </c>
       <c r="V355">
-        <v>-343.56</v>
+        <v>-687.12</v>
       </c>
       <c r="W355">
         <v>-343.56</v>
@@ -17449,11 +17395,8 @@
       <c r="E385">
         <v>-34120.92</v>
       </c>
-      <c r="V385">
-        <v>-2843.41</v>
-      </c>
       <c r="W385">
-        <v>-2843.41</v>
+        <v>-5686.82</v>
       </c>
       <c r="X385">
         <v>-2843.41</v>
@@ -19137,14 +19080,8 @@
       <c r="E425">
         <v>-24965.88</v>
       </c>
-      <c r="V425">
-        <v>-2080.49</v>
-      </c>
-      <c r="W425">
-        <v>-2080.49</v>
-      </c>
       <c r="X425">
-        <v>-2080.49</v>
+        <v>-6241.47</v>
       </c>
       <c r="Y425">
         <v>-2080.49</v>
@@ -19190,14 +19127,8 @@
       <c r="E426">
         <v>-30909.84</v>
       </c>
-      <c r="V426">
-        <v>-2575.82</v>
-      </c>
-      <c r="W426">
-        <v>-2575.82</v>
-      </c>
       <c r="X426">
-        <v>-2575.82</v>
+        <v>-7727.46</v>
       </c>
       <c r="Y426">
         <v>-2575.82</v>
@@ -20825,7 +20756,7 @@
       <c r="E459">
         <v>-8140.97</v>
       </c>
-      <c r="W459">
+      <c r="Y459">
         <v>-8140.97</v>
       </c>
     </row>
@@ -22704,14 +22635,8 @@
       <c r="E500">
         <v>-2538.66</v>
       </c>
-      <c r="X500">
-        <v>-423.11</v>
-      </c>
-      <c r="Y500">
-        <v>-423.11</v>
-      </c>
       <c r="Z500">
-        <v>-423.11</v>
+        <v>-1269.33</v>
       </c>
       <c r="AA500">
         <v>-423.11</v>
@@ -22739,7 +22664,7 @@
       <c r="E501">
         <v>-17958.09</v>
       </c>
-      <c r="Y501">
+      <c r="Z501">
         <v>-17958.09</v>
       </c>
     </row>
@@ -24641,11 +24566,8 @@
       <c r="E540">
         <v>-20669.28</v>
       </c>
-      <c r="Z540">
-        <v>-1722.44</v>
-      </c>
       <c r="AA540">
-        <v>-1722.44</v>
+        <v>-3444.88</v>
       </c>
       <c r="AB540">
         <v>-1722.44</v>
@@ -29154,11 +29076,8 @@
       <c r="E638">
         <v>-835.28</v>
       </c>
-      <c r="AB638">
-        <v>-417.64</v>
-      </c>
       <c r="AC638">
-        <v>-417.64</v>
+        <v>-835.28</v>
       </c>
     </row>
     <row r="639">
@@ -29177,11 +29096,8 @@
       <c r="E639">
         <v>-18960.84</v>
       </c>
-      <c r="AB639">
-        <v>-1580.07</v>
-      </c>
       <c r="AC639">
-        <v>-1580.07</v>
+        <v>-3160.14</v>
       </c>
       <c r="AD639">
         <v>-1580.07</v>
@@ -29230,11 +29146,8 @@
       <c r="E640">
         <v>-646.47</v>
       </c>
-      <c r="AB640">
-        <v>-215.49</v>
-      </c>
       <c r="AC640">
-        <v>-215.49</v>
+        <v>-430.98</v>
       </c>
       <c r="AD640">
         <v>-215.49</v>
@@ -29256,11 +29169,8 @@
       <c r="E641">
         <v>-5223.9</v>
       </c>
-      <c r="AB641">
-        <v>-522.39</v>
-      </c>
       <c r="AC641">
-        <v>-522.39</v>
+        <v>-1044.78</v>
       </c>
       <c r="AD641">
         <v>-522.39</v>
@@ -29303,14 +29213,8 @@
       <c r="E642">
         <v>-23360.64</v>
       </c>
-      <c r="AA642">
-        <v>-1946.72</v>
-      </c>
-      <c r="AB642">
-        <v>-1946.72</v>
-      </c>
       <c r="AC642">
-        <v>-1946.72</v>
+        <v>-5840.16</v>
       </c>
       <c r="AD642">
         <v>-1946.72</v>
@@ -31439,7 +31343,7 @@
       <c r="E687">
         <v>-17170.66</v>
       </c>
-      <c r="AB687">
+      <c r="AD687">
         <v>-17170.66</v>
       </c>
     </row>
@@ -31459,11 +31363,8 @@
       <c r="E688">
         <v>-77718.24</v>
       </c>
-      <c r="AC688">
-        <v>-3238.26</v>
-      </c>
       <c r="AD688">
-        <v>-3238.26</v>
+        <v>-6476.52</v>
       </c>
       <c r="AE688">
         <v>-3238.26</v>
@@ -31548,7 +31449,7 @@
       <c r="E689">
         <v>-10343.67</v>
       </c>
-      <c r="AC689">
+      <c r="AD689">
         <v>-10343.67</v>
       </c>
     </row>
@@ -31568,14 +31469,8 @@
       <c r="E690">
         <v>-40622.52</v>
       </c>
-      <c r="AB690">
-        <v>-3385.21</v>
-      </c>
-      <c r="AC690">
-        <v>-3385.21</v>
-      </c>
       <c r="AD690">
-        <v>-3385.21</v>
+        <v>-10155.63</v>
       </c>
       <c r="AE690">
         <v>-3385.21</v>
@@ -33213,7 +33108,7 @@
       <c r="E722">
         <v>-20674.89</v>
       </c>
-      <c r="AC722">
+      <c r="AE722">
         <v>-20674.89</v>
       </c>
     </row>
@@ -35245,14 +35140,8 @@
       <c r="E766">
         <v>-27438.84</v>
       </c>
-      <c r="AD766">
-        <v>-2286.57</v>
-      </c>
-      <c r="AE766">
-        <v>-2286.57</v>
-      </c>
       <c r="AF766">
-        <v>-2286.57</v>
+        <v>-6859.71</v>
       </c>
       <c r="AG766">
         <v>-2286.57</v>
@@ -35298,14 +35187,8 @@
       <c r="E767">
         <v>-1893.6</v>
       </c>
-      <c r="AD767">
-        <v>-210.4</v>
-      </c>
-      <c r="AE767">
-        <v>-210.4</v>
-      </c>
       <c r="AF767">
-        <v>-210.4</v>
+        <v>-631.2</v>
       </c>
       <c r="AG767">
         <v>-210.4</v>
@@ -35342,14 +35225,8 @@
       <c r="E768">
         <v>-13687.56</v>
       </c>
-      <c r="AD768">
-        <v>-1140.63</v>
-      </c>
-      <c r="AE768">
-        <v>-1140.63</v>
-      </c>
       <c r="AF768">
-        <v>-1140.63</v>
+        <v>-3421.89</v>
       </c>
       <c r="AG768">
         <v>-1140.63</v>
@@ -37346,11 +37223,8 @@
       <c r="E810">
         <v>-19847.04</v>
       </c>
-      <c r="AF810">
-        <v>-1653.92</v>
-      </c>
       <c r="AG810">
-        <v>-1653.92</v>
+        <v>-3307.84</v>
       </c>
       <c r="AH810">
         <v>-1653.92</v>
@@ -37399,7 +37273,7 @@
       <c r="E811">
         <v>-16084.93</v>
       </c>
-      <c r="AE811">
+      <c r="AG811">
         <v>-16084.93</v>
       </c>
     </row>
@@ -37419,14 +37293,8 @@
       <c r="E812">
         <v>-42144.6</v>
       </c>
-      <c r="AE812">
-        <v>-3512.05</v>
-      </c>
-      <c r="AF812">
-        <v>-3512.05</v>
-      </c>
       <c r="AG812">
-        <v>-3512.05</v>
+        <v>-10536.15</v>
       </c>
       <c r="AH812">
         <v>-3512.05</v>
@@ -39236,7 +39104,7 @@
       <c r="E852">
         <v>-5473.99</v>
       </c>
-      <c r="AG852">
+      <c r="AH852">
         <v>-5473.99</v>
       </c>
     </row>
@@ -41500,11 +41368,8 @@
       <c r="E901">
         <v>-4497.12</v>
       </c>
-      <c r="AH901">
-        <v>-374.76</v>
-      </c>
       <c r="AI901">
-        <v>-374.76</v>
+        <v>-749.52</v>
       </c>
       <c r="AJ901">
         <v>-374.76</v>
@@ -44695,7 +44560,7 @@
       <c r="E973">
         <v>-17481.73</v>
       </c>
-      <c r="AI973">
+      <c r="AK973">
         <v>-17481.73</v>
       </c>
     </row>
@@ -44715,11 +44580,8 @@
       <c r="E974">
         <v>-24450.84</v>
       </c>
-      <c r="AJ974">
-        <v>-2037.57</v>
-      </c>
       <c r="AK974">
-        <v>-2037.57</v>
+        <v>-4075.14</v>
       </c>
       <c r="AL974">
         <v>-2037.57</v>
@@ -46906,14 +46768,8 @@
       <c r="E1021">
         <v>-38091.35</v>
       </c>
-      <c r="AJ1021">
-        <v>-3462.85</v>
-      </c>
-      <c r="AK1021">
-        <v>-3462.85</v>
-      </c>
       <c r="AL1021">
-        <v>-3462.85</v>
+        <v>-10388.55</v>
       </c>
       <c r="AM1021">
         <v>-3462.85</v>
@@ -49125,11 +48981,8 @@
       <c r="E1073">
         <v>-3341.64</v>
       </c>
-      <c r="AL1073">
-        <v>-278.47</v>
-      </c>
       <c r="AM1073">
-        <v>-278.47</v>
+        <v>-556.94</v>
       </c>
       <c r="AN1073">
         <v>-278.47</v>
@@ -49222,7 +49075,7 @@
       <c r="E1075">
         <v>-20176.88</v>
       </c>
-      <c r="AK1075">
+      <c r="AM1075">
         <v>-20176.88</v>
       </c>
     </row>
@@ -49242,14 +49095,8 @@
       <c r="E1076">
         <v>-46251.36</v>
       </c>
-      <c r="AK1076">
-        <v>-3854.28</v>
-      </c>
-      <c r="AL1076">
-        <v>-3854.28</v>
-      </c>
       <c r="AM1076">
-        <v>-3854.28</v>
+        <v>-11562.84</v>
       </c>
       <c r="AN1076">
         <v>-3854.28</v>
@@ -49348,14 +49195,8 @@
       <c r="E1078">
         <v>-18183.48</v>
       </c>
-      <c r="AK1078">
-        <v>-1515.29</v>
-      </c>
-      <c r="AL1078">
-        <v>-1515.29</v>
-      </c>
       <c r="AM1078">
-        <v>-1515.29</v>
+        <v>-4545.87</v>
       </c>
       <c r="AN1078">
         <v>-1515.29</v>
@@ -49430,11 +49271,8 @@
       <c r="E1080">
         <v>-27298.44</v>
       </c>
-      <c r="AL1080">
-        <v>-2274.87</v>
-      </c>
       <c r="AM1080">
-        <v>-2274.87</v>
+        <v>-4549.74</v>
       </c>
       <c r="AN1080">
         <v>-2274.87</v>

</xml_diff>